<commit_message>
feat: complete enterprise UI improvements and bug fixes
</commit_message>
<xml_diff>
--- a/src/assets/project-tracker/HAATZA_Test_Cases.xlsx
+++ b/src/assets/project-tracker/HAATZA_Test_Cases.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H36"/>
+  <dimension ref="A1:H50"/>
   <cols>
     <col min="1" max="1" width="20.83203125" customWidth="1"/>
     <col min="2" max="2" width="25.83203125" customWidth="1"/>
@@ -1141,22 +1141,22 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>Access Control</v>
+        <v>Operations</v>
       </c>
       <c r="B29" t="str">
-        <v>TC-AC-01</v>
+        <v>TC-OP-01</v>
       </c>
       <c r="C29" t="str">
-        <v>Module Access Blockage</v>
+        <v>Order Picking Workspace Validation</v>
       </c>
       <c r="D29" t="str">
-        <v>Login as restricted role (e.g. Human Resources), attempt to visit `/finance/gst-reports`</v>
+        <v>Navigate to Operations -&gt; Order Picking, select picklist #PK-102, scan barcode and enter bin locator code.</v>
       </c>
       <c r="E29" t="str">
-        <v>Router intercepts navigation and redirects user to Access Denied (/unauthorized) page.</v>
+        <v>Pick status updates to Picked and item moves to packing bay in ledger.</v>
       </c>
       <c r="F29" t="str">
-        <v>Completed</v>
+        <v>Pending</v>
       </c>
       <c r="G29" t="str">
         <v>Pending</v>
@@ -1167,22 +1167,22 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>Access Control</v>
+        <v>Operations</v>
       </c>
       <c r="B30" t="str">
-        <v>TC-AC-02</v>
+        <v>TC-OP-02</v>
       </c>
       <c r="C30" t="str">
-        <v>Role-Page Matrix Validation</v>
+        <v>Generate Shift Assignment</v>
       </c>
       <c r="D30" t="str">
-        <v>Run diagnostic simulation for restricted roles in IT &gt; Role &amp; Permissions QA console</v>
+        <v>Open Shift Management, enter worker name, select role, select allocation, and click Generate Shift Slot.</v>
       </c>
       <c r="E30" t="str">
-        <v>Consoles scans all 106 pages, matching accessible and restricted lists to matrix schema with 100% accuracy.</v>
+        <v>Worker is added to Daily Shift Board with status Present.</v>
       </c>
       <c r="F30" t="str">
-        <v>Completed</v>
+        <v>Pending</v>
       </c>
       <c r="G30" t="str">
         <v>Pending</v>
@@ -1193,22 +1193,22 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>Access Control</v>
+        <v>Inventory</v>
       </c>
       <c r="B31" t="str">
-        <v>TC-AC-03</v>
+        <v>TC-INV-01</v>
       </c>
       <c r="C31" t="str">
-        <v>Sidebar Node Visibility</v>
+        <v>Stock Inward &amp; Putaway Flow</v>
       </c>
       <c r="D31" t="str">
-        <v>Login as restricted role (e.g. Marketing), inspect the left navigation sidebar</v>
+        <v>Navigate to Inventory -&gt; Stock Inward, enter product barcode, enter received quantity (100 units), bin ID, and click Submit Putaway.</v>
       </c>
       <c r="E31" t="str">
-        <v>Only the Marketing group and general Settings/Support directories are visible; other role folders are hidden.</v>
+        <v>Stock level for specified SKU increments by 100 units in the Inventory Management table.</v>
       </c>
       <c r="F31" t="str">
-        <v>Completed</v>
+        <v>Pending</v>
       </c>
       <c r="G31" t="str">
         <v>Pending</v>
@@ -1219,22 +1219,22 @@
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>Access Control</v>
+        <v>Inventory</v>
       </c>
       <c r="B32" t="str">
-        <v>TC-AC-04</v>
+        <v>TC-INV-02</v>
       </c>
       <c r="C32" t="str">
-        <v>Route Protection Guards</v>
+        <v>Expiry Tracker Alerts</v>
       </c>
       <c r="D32" t="str">
-        <v>Directly enter route URL of restricted page (e.g. `/hr/payroll`) into address bar</v>
+        <v>Open Expiry Management, verify threshold warning display and expired batches highlighting.</v>
       </c>
       <c r="E32" t="str">
-        <v>RouteGuard intercepts rendering, validates lack of permission, and forces redirect to `/unauthorized`.</v>
+        <v>System lists batches expiring within threshold in red, blocking them from picker lists.</v>
       </c>
       <c r="F32" t="str">
-        <v>Completed</v>
+        <v>Pending</v>
       </c>
       <c r="G32" t="str">
         <v>Pending</v>
@@ -1245,22 +1245,22 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>Access Control</v>
+        <v>Purchase</v>
       </c>
       <c r="B33" t="str">
-        <v>TC-AC-05</v>
+        <v>TC-PUR-01</v>
       </c>
       <c r="C33" t="str">
-        <v>Action Permission Restrictions</v>
+        <v>Auto Requisition Generation</v>
       </c>
       <c r="D33" t="str">
-        <v>Access page as restricted role (e.g. Finance &gt; GST Reports), attempt restricted CRUD action (e.g. Delete)</v>
+        <v>Navigate to Purchase Dashboard, click Run Auto-Replenish Engine.</v>
       </c>
       <c r="E33" t="str">
-        <v>Delete action button is disabled with lock indicator, and attempts log 403 Forbidden in REST console.</v>
+        <v>System scans inventory and auto-generates Purchase Requests for low stock items.</v>
       </c>
       <c r="F33" t="str">
-        <v>Completed</v>
+        <v>Pending</v>
       </c>
       <c r="G33" t="str">
         <v>Pending</v>
@@ -1271,22 +1271,22 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>Access Control</v>
+        <v>Purchase</v>
       </c>
       <c r="B34" t="str">
-        <v>TC-AC-06</v>
+        <v>TC-PUR-02</v>
       </c>
       <c r="C34" t="str">
-        <v>Admin Override Mode</v>
+        <v>Goods Receipt (GRN) Temperature Control</v>
       </c>
       <c r="D34" t="str">
-        <v>Login as Administrator/Admin, verify sidebar, navigation, and page action availability</v>
+        <v>Attempt to register a Dairy shipment with Probe Temp 5.5°C (Limit &lt;= 4.5°C).</v>
       </c>
       <c r="E34" t="str">
-        <v>All 11 role-based folders and 106 pages are visible; all CRUD action buttons (Create, Edit, Delete, Export, etc.) are enabled.</v>
+        <v>Submission blocks with warning: 'Dairy temperature cannot exceed 4.5°C'.</v>
       </c>
       <c r="F34" t="str">
-        <v>Completed</v>
+        <v>Pending</v>
       </c>
       <c r="G34" t="str">
         <v>Pending</v>
@@ -1297,22 +1297,22 @@
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>Access Control</v>
+        <v>Logistics &amp; Delivery</v>
       </c>
       <c r="B35" t="str">
-        <v>TC-AC-07</v>
+        <v>TC-LOG-01</v>
       </c>
       <c r="C35" t="str">
-        <v>Unauthorized Guest Blockage</v>
+        <v>Delivery Rider Assignment</v>
       </c>
       <c r="D35" t="str">
-        <v>Open a fresh incognito window and attempt to access dashboard URL (`/`) directly</v>
+        <v>Navigate to Logistics &amp; Delivery -&gt; Delivery Assignment, select dispatch manifest, choose Rider, and click Assign &amp; Notify.</v>
       </c>
       <c r="E35" t="str">
-        <v>System detects unauthenticated state and redirects guest immediately to the Login screen.</v>
+        <v>Manifest transitions to Assigned and order status is updated.</v>
       </c>
       <c r="F35" t="str">
-        <v>Completed</v>
+        <v>Pending</v>
       </c>
       <c r="G35" t="str">
         <v>Pending</v>
@@ -1323,33 +1323,397 @@
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>Access Control</v>
+        <v>Logistics &amp; Delivery</v>
       </c>
       <c r="B36" t="str">
-        <v>TC-AC-08</v>
+        <v>TC-LOG-02</v>
       </c>
       <c r="C36" t="str">
-        <v>Session Refresher Sync</v>
+        <v>Route Optimization Check</v>
       </c>
       <c r="D36" t="str">
-        <v>Switch active role on the workspace connection setup screen</v>
+        <v>Open Route Management, input multiple destination drops, and click Generate Route.</v>
       </c>
       <c r="E36" t="str">
-        <v>Accessible pages list and active session variables are wiped and reconstructed with zero permission leaks.</v>
+        <v>System plots the optimized route listing total distance and travel duration.</v>
       </c>
       <c r="F36" t="str">
-        <v>Completed</v>
+        <v>Pending</v>
       </c>
       <c r="G36" t="str">
         <v>Pending</v>
       </c>
       <c r="H36" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>Customer Support</v>
+      </c>
+      <c r="B37" t="str">
+        <v>TC-CS-01</v>
+      </c>
+      <c r="C37" t="str">
+        <v>Customer Ticket Creation</v>
+      </c>
+      <c r="D37" t="str">
+        <v>Open Customer Tickets, click Create Ticket, enter order #, select category, enter description, and submit.</v>
+      </c>
+      <c r="E37" t="str">
+        <v>Ticket is created with status Open and routed to support queue.</v>
+      </c>
+      <c r="F37" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="G37" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="H37" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>Customer Support</v>
+      </c>
+      <c r="B38" t="str">
+        <v>TC-CS-02</v>
+      </c>
+      <c r="C38" t="str">
+        <v>Order Lookup &amp; Refund Request</v>
+      </c>
+      <c r="D38" t="str">
+        <v>Open Order Lookup, search by customer email, select order, and click Initiate Refund.</v>
+      </c>
+      <c r="E38" t="str">
+        <v>Order details load and refund request is submitted to Finance as Pending Approval.</v>
+      </c>
+      <c r="F38" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="G38" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="H38" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>Sales &amp; Business</v>
+      </c>
+      <c r="B39" t="str">
+        <v>TC-SB-01</v>
+      </c>
+      <c r="C39" t="str">
+        <v>Merchant Partner Onboarding</v>
+      </c>
+      <c r="D39" t="str">
+        <v>Navigate to Sales &amp; Business -&gt; Merchant Management, click Register Merchant, enter business/tax details, and click Onboard.</v>
+      </c>
+      <c r="E39" t="str">
+        <v>Merchant account is created and visible in Partner Management.</v>
+      </c>
+      <c r="F39" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="G39" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="H39" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v>Sales &amp; Business</v>
+      </c>
+      <c r="B40" t="str">
+        <v>TC-SB-02</v>
+      </c>
+      <c r="C40" t="str">
+        <v>Expansion Planning Opportunity Tracker</v>
+      </c>
+      <c r="D40" t="str">
+        <v>Open Expansion Planning, click Add Proposal, specify location, estimated demand tier, and launch cost.</v>
+      </c>
+      <c r="E40" t="str">
+        <v>Proposal is listed in active opportunities list.</v>
+      </c>
+      <c r="F40" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="G40" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="H40" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v>Marketing</v>
+      </c>
+      <c r="B41" t="str">
+        <v>TC-MKT-01</v>
+      </c>
+      <c r="C41" t="str">
+        <v>Create Coupon Code Promotion</v>
+      </c>
+      <c r="D41" t="str">
+        <v>Navigate to Coupons &amp; Offers, click Create Coupon, enter promo details, discount rules, and save.</v>
+      </c>
+      <c r="E41" t="str">
+        <v>Coupon is registered and active for checkout validations.</v>
+      </c>
+      <c r="F41" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="G41" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="H41" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <v>Marketing</v>
+      </c>
+      <c r="B42" t="str">
+        <v>TC-MKT-02</v>
+      </c>
+      <c r="C42" t="str">
+        <v>Push Notification Campaign Segment</v>
+      </c>
+      <c r="D42" t="str">
+        <v>Open Push Notifications, choose Audience Segment, enter Title/Body, and click Send Blast.</v>
+      </c>
+      <c r="E42" t="str">
+        <v>System dispatches push notification to matched customer profiles.</v>
+      </c>
+      <c r="F42" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="G42" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="H42" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="str">
+        <v>Finance &amp; Accounts</v>
+      </c>
+      <c r="B43" t="str">
+        <v>TC-FIN-01</v>
+      </c>
+      <c r="C43" t="str">
+        <v>Vendor Payments Settlements</v>
+      </c>
+      <c r="D43" t="str">
+        <v>Navigate to Vendor Payments, select invoice, verify matched GRN, enter transaction reference, and click Settle Payment.</v>
+      </c>
+      <c r="E43" t="str">
+        <v>Invoice status shifts to Paid and ledger balances.</v>
+      </c>
+      <c r="F43" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="G43" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="H43" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="str">
+        <v>Finance &amp; Accounts</v>
+      </c>
+      <c r="B44" t="str">
+        <v>TC-FIN-02</v>
+      </c>
+      <c r="C44" t="str">
+        <v>GST Audit Report Generation</v>
+      </c>
+      <c r="D44" t="str">
+        <v>Open GST Reports, select month, and click Generate Report.</v>
+      </c>
+      <c r="E44" t="str">
+        <v>GST liability is computed and available for Excel/PDF download.</v>
+      </c>
+      <c r="F44" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="G44" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="H44" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="str">
+        <v>Human Resources</v>
+      </c>
+      <c r="B45" t="str">
+        <v>TC-HR-01</v>
+      </c>
+      <c r="C45" t="str">
+        <v>Employee Attendance Verification</v>
+      </c>
+      <c r="D45" t="str">
+        <v>Open Attendance, select Employee ID, enter check-in time, and confirm.</v>
+      </c>
+      <c r="E45" t="str">
+        <v>Employee status updates to Present and total working hours recalculate.</v>
+      </c>
+      <c r="F45" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="G45" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="H45" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="str">
+        <v>Human Resources</v>
+      </c>
+      <c r="B46" t="str">
+        <v>TC-HR-02</v>
+      </c>
+      <c r="C46" t="str">
+        <v>Leave Request Submission</v>
+      </c>
+      <c r="D46" t="str">
+        <v>Navigate to Leave Management, click Request Leave, specify dates/type, and submit.</v>
+      </c>
+      <c r="E46" t="str">
+        <v>Leave request is logged with status Pending Manager Approval.</v>
+      </c>
+      <c r="F46" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="G46" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="H46" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="str">
+        <v>Information Technology</v>
+      </c>
+      <c r="B47" t="str">
+        <v>TC-IT-01</v>
+      </c>
+      <c r="C47" t="str">
+        <v>Modify User Role Permissions</v>
+      </c>
+      <c r="D47" t="str">
+        <v>Navigate to Role &amp; Permissions, select user, toggle page permission, and click Save Settings.</v>
+      </c>
+      <c r="E47" t="str">
+        <v>User permissions list is updated, enforcing new access on next request.</v>
+      </c>
+      <c r="F47" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="G47" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="H47" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="str">
+        <v>Information Technology</v>
+      </c>
+      <c r="B48" t="str">
+        <v>TC-IT-02</v>
+      </c>
+      <c r="C48" t="str">
+        <v>API Log Traversal</v>
+      </c>
+      <c r="D48" t="str">
+        <v>Open API Logs, search for error status code 500, check details.</v>
+      </c>
+      <c r="E48" t="str">
+        <v>Logs are filtered displaying payload and response latency.</v>
+      </c>
+      <c r="F48" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="G48" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="H48" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="str">
+        <v>Administration</v>
+      </c>
+      <c r="B49" t="str">
+        <v>TC-ADM-01</v>
+      </c>
+      <c r="C49" t="str">
+        <v>Asset Allocation Log</v>
+      </c>
+      <c r="D49" t="str">
+        <v>Navigate to Asset Management, click Allocate Asset, select asset scanner, select assignee, and submit.</v>
+      </c>
+      <c r="E49" t="str">
+        <v>Asset status changes to Allocated and custody record is saved.</v>
+      </c>
+      <c r="F49" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="G49" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="H49" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="str">
+        <v>Administration</v>
+      </c>
+      <c r="B50" t="str">
+        <v>TC-ADM-02</v>
+      </c>
+      <c r="C50" t="str">
+        <v>Facility Maintenance Request</v>
+      </c>
+      <c r="D50" t="str">
+        <v>Open Facility Management, click Log Maintenance Job, specify area/priority, enter description, and submit.</v>
+      </c>
+      <c r="E50" t="str">
+        <v>Maintenance ticket is registered and email alert sent to service provider.</v>
+      </c>
+      <c r="F50" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="G50" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="H50" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H36"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H50"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>